<commit_message>
Connector BOM workbook: merge front-left/front-right into one front branch (same symmetric part, qty 2)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MdxDfxB8wg2Ht2aZSuwqK
</commit_message>
<xml_diff>
--- a/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
+++ b/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="82">
   <si>
     <t xml:space="preserve">MERITAGE FLAT CONNECTOR SYSTEM · BOM REWORK BY BRANCH</t>
   </si>
@@ -43,7 +43,7 @@
     <t xml:space="preserve">LEGEND:  orange = current state (problem) · green = new state (target) · blue-gray = deliverables to create · yellow cells = fill in Owner / Status / dates</t>
   </si>
   <si>
-    <t xml:space="preserve">BRANCH 1 · FRONT LEFT CONNECTOR   ·   Config 1 (front, same part both front corners)</t>
+    <t xml:space="preserve">BRANCH 1 · FRONT CONNECTORS (BOTH CORNERS, ONE PART)   ·   Config 1: symmetric part, qty 2 per unit, no left/right versions and no flipping</t>
   </si>
   <si>
     <t xml:space="preserve">CURRENT BOM (as shipped today)</t>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 1 (front): unique P/N, matches the seat-frame assembly drawing and TU-530 Rev A</t>
   </si>
   <si>
-    <t xml:space="preserve">Qty 2 per unit across both front corners</t>
+    <t xml:space="preserve">One P/N covers both front corners</t>
   </si>
   <si>
     <t xml:space="preserve">Pre-fitted screw</t>
@@ -157,66 +157,36 @@
     <t xml:space="preserve">[Engineering]  Engineering validation of screw 1012919 as the released spec</t>
   </si>
   <si>
-    <t xml:space="preserve">BRANCH 2 · FRONT RIGHT CONNECTOR   ·   Config 1 (front, same part both front corners)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same generic part and wrong-drawing situation as front left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shares the front configuration; no left/right issue at the front</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrives installed; wrong, swapped by the operator every time</t>
+    <t xml:space="preserve">BRANCH 2 · BACK LEFT CONNECTOR   ·   Config 2 (back left, orientation-specific)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(shared P/N)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Back-left and back-right SHARE one part number today; drawings show wrong P/N 1012553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The two back configurations are physically different but undistinguished</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012934</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrives installed; wrong, operator swaps it</t>
   </si>
   <si>
     <t xml:space="preserve">Part of the 11:40/unit rework</t>
   </si>
   <si>
+    <t xml:space="preserve">40204</t>
+  </si>
+  <si>
     <t xml:space="preserve">What the operator actually installs</t>
   </si>
   <si>
     <t xml:space="preserve">Unofficial, not on BOM</t>
   </si>
   <si>
-    <t xml:space="preserve">Same Config 1 P/N as front left (the front part is symmetric)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Covered by the qty-2 front line on the BOM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ships installed by the supplier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same validation as front left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Note]  No separate deliverables: fully covered by the Front Left branch (same P/N 1015301, same drawing, same PO line)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[BOM]  Verify the BOM front line reads qty 2 so both corners are covered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BRANCH 3 · BACK LEFT CONNECTOR   ·   Config 2 (back left, orientation-specific)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(shared P/N)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Back-left and back-right SHARE one part number today; drawings show wrong P/N 1012553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The two back configurations are physically different but undistinguished</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1012934</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrives installed; wrong, operator swaps it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40204</t>
-  </si>
-  <si>
     <t xml:space="preserve">Orientation</t>
   </si>
   <si>
@@ -259,7 +229,7 @@
     <t xml:space="preserve">[Engineering]  Engineering validation of screw 40204 as the released spec</t>
   </si>
   <si>
-    <t xml:space="preserve">BRANCH 4 · BACK RIGHT CONNECTOR   ·   Config 3 (back right, orientation-specific)</t>
+    <t xml:space="preserve">BRANCH 3 · BACK RIGHT CONNECTOR   ·   Config 3 (back right, orientation-specific)</t>
   </si>
   <si>
     <t xml:space="preserve">Shares a part number with back-left today; drawings show wrong P/N 1012553</t>
@@ -905,7 +875,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1025,7 +995,7 @@
         <v>17</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="16" t="s">
         <v>18</v>
@@ -1045,7 +1015,7 @@
         <v>21</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>22</v>
@@ -1065,7 +1035,7 @@
         <v>25</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="16" t="s">
         <v>26</v>
@@ -1115,7 +1085,7 @@
         <v>31</v>
       </c>
       <c r="E18" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="21" t="s">
         <v>32</v>
@@ -1135,7 +1105,7 @@
         <v>34</v>
       </c>
       <c r="E19" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>35</v>
@@ -1224,14 +1194,14 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
@@ -1271,16 +1241,16 @@
         <v>15</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E30" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1291,16 +1261,16 @@
         <v>19</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E31" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1311,134 +1281,140 @@
         <v>23</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E32" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B35" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C35" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D35" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E35" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="F35" s="13" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B35" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D35" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="E35" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="21" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="E36" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B37" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="E36" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="22" t="s">
+      <c r="C37" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E37" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="22"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="22"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
+      <c r="B38" s="22"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="22"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B39" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13" t="s">
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F39" s="13" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C40" s="24"/>
       <c r="D40" s="24"/>
@@ -1447,267 +1423,267 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B42" s="26"/>
-      <c r="C42" s="26"/>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
+    <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" s="24"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43" s="24"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B47" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="C47" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D47" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E44" s="12" t="s">
+      <c r="E47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F44" s="13" t="s">
+      <c r="F47" s="13" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B45" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B46" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C46" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="D46" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B47" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C47" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D47" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E47" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="16" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D48" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D49" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D50" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B48" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="C48" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="D48" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F48" s="16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17" t="s">
+      <c r="B51" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D51" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F51" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="12" t="s">
+      <c r="B52" s="17"/>
+      <c r="C52" s="17"/>
+      <c r="D52" s="17"/>
+      <c r="E52" s="17"/>
+      <c r="F52" s="17"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B53" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C50" s="13" t="s">
+      <c r="C53" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="D53" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="E53" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F50" s="13" t="s">
+      <c r="F53" s="13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B51" s="19" t="s">
+    <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C51" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="D51" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="E51" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18" t="n">
+      <c r="C54" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="E54" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B52" s="19" t="s">
+      <c r="B55" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C52" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="E52" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="21" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="22" t="s">
+      <c r="C55" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E55" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B53" s="22"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="22"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12" t="s">
+      <c r="B56" s="22"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B54" s="13" t="s">
+      <c r="B57" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13" t="s">
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F54" s="13" t="s">
+      <c r="F57" s="13" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B55" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="C55" s="24"/>
-      <c r="D55" s="24"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B56" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="C56" s="24"/>
-      <c r="D56" s="24"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B57" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="C57" s="24"/>
-      <c r="D57" s="24"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="25" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B58" s="24" t="s">
         <v>78</v>
@@ -1719,280 +1695,50 @@
         <v>41</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="27" t="s">
+    <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B59" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B60" s="27"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="27"/>
-      <c r="E60" s="27"/>
-      <c r="F60" s="27"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B62" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C62" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D62" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C63" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="D63" s="15" t="s">
+      <c r="C59" s="24"/>
+      <c r="D59" s="24"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B60" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="E63" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F63" s="16" t="s">
+      <c r="C60" s="24"/>
+      <c r="D60" s="24"/>
+      <c r="E60" s="25"/>
+      <c r="F60" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" s="24" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B64" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="D64" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="E64" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F64" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B65" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C65" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D65" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E65" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F65" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B66" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="C66" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="D66" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="E66" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F66" s="16" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B67" s="17"/>
-      <c r="C67" s="17"/>
-      <c r="D67" s="17"/>
-      <c r="E67" s="17"/>
-      <c r="F67" s="17"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B68" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C68" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D68" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F68" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B69" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C69" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="D69" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="E69" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C70" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D70" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="E70" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" s="21" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B71" s="22"/>
-      <c r="C71" s="22"/>
-      <c r="D71" s="22"/>
-      <c r="E71" s="22"/>
-      <c r="F71" s="22"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B72" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C72" s="13"/>
-      <c r="D72" s="13"/>
-      <c r="E72" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F72" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B73" s="24" t="s">
-        <v>88</v>
-      </c>
-      <c r="C73" s="24"/>
-      <c r="D73" s="24"/>
-      <c r="E73" s="25"/>
-      <c r="F73" s="25" t="s">
+      <c r="C61" s="24"/>
+      <c r="D61" s="24"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B74" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="C74" s="24"/>
-      <c r="D74" s="24"/>
-      <c r="E74" s="25"/>
-      <c r="F74" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B75" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="C75" s="24"/>
-      <c r="D75" s="24"/>
-      <c r="E75" s="25"/>
-      <c r="F75" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="B76" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="C76" s="24"/>
-      <c r="D76" s="24"/>
-      <c r="E76" s="25"/>
-      <c r="F76" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="30">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A8:F8"/>
@@ -2007,29 +1753,22 @@
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="B39:D39"/>
     <mergeCell ref="B40:D40"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="B57:D57"/>
     <mergeCell ref="B58:D58"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B74:D74"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B61:D61"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Connector workbook: 1012553 is the valid bare component; differentiate at ASSEMBLY level
Reframed per floor insight: 1012553 is the bare connector piece, shared
by every position and unchanged. The gap is the assembly level: three
assemblies (1015301 = 1012553+1012919 front x2; 1015302 = +40204 LH;
1016592 = +40204 RH) need defining/ordering. Removed 'supersedes
1012553' and wrong-P/N framing; new-BOM sections show assembly with its
components; deliverables are assembly drawings + BOM lines + order-by-
assembly-P/N supplier instructions.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MdxDfxB8wg2Ht2aZSuwqK
</commit_message>
<xml_diff>
--- a/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
+++ b/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="89">
   <si>
     <t xml:space="preserve">MERITAGE FLAT CONNECTOR SYSTEM · BOM REWORK BY BRANCH</t>
   </si>
   <si>
-    <t xml:space="preserve">Root cause: three real connector configurations exist, the BOM lists two, and the connector drawings carry P/N 1012553 (matches nothing). Supplier ships one generic part; the line hand-reworks every connector. Scope: part numbers and pre-fitted screws (ECN Items A and B), 07/2026.</t>
+    <t xml:space="preserve">How to read this: 1012553 is the BARE connector piece (shared component, used in every position, unchanged). The differentiation happens one level up, at the ASSEMBLY: bare connector + the right screw + the right orientation = three distinct assemblies (1015301 front, 1015302 back-left, 1016592 back-right). Today the supplier effectively ships ONE generic assembly, so the line swaps screws and flips orientation by hand. Scope: define and order the three assemblies, 07/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Labor recovered per unit (min)</t>
@@ -67,16 +67,28 @@
     <t xml:space="preserve">Problem / note</t>
   </si>
   <si>
-    <t xml:space="preserve">Flat connector, generic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(no unique P/N)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One generic configuration for all positions; connector drawings show P/N 1012553, which matches neither the BOM nor the floor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOM lists only 2 connector types for 3 real configurations</t>
+    <t xml:space="preserve">Bare connector (component)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1012553</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The connector piece itself, no screws. Shared by every position; this part is CORRECT and does not change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK as-is: the shared base component</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assembly, as shipped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(generic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supplier assembles the bare connector with screw 40200; no front-specific assembly P/N is ordered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The generic assembly is what forces the rework</t>
   </si>
   <si>
     <t xml:space="preserve">Screw, as shipped</t>
@@ -85,7 +97,7 @@
     <t xml:space="preserve">40200</t>
   </si>
   <si>
-    <t xml:space="preserve">Arrives installed; WRONG for this position, operator removes it on every connector</t>
+    <t xml:space="preserve">Installed by the supplier; wrong for the front position, operator removes it on every connector</t>
   </si>
   <si>
     <t xml:space="preserve">Removed and replaced on the line (part of the 11:40/unit rework)</t>
@@ -100,7 +112,7 @@
     <t xml:space="preserve">What the operator actually installs (working baseline, not on BOM)</t>
   </si>
   <si>
-    <t xml:space="preserve">Unofficial: consumed on the line but not in the connector BOM</t>
+    <t xml:space="preserve">Unofficial: consumed on the line but not in the assembly BOM</t>
   </si>
   <si>
     <t xml:space="preserve">NEW BOM (ships pre-configured)</t>
@@ -109,22 +121,31 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Connector assembly</t>
+    <t xml:space="preserve">Connector ASSEMBLY</t>
   </si>
   <si>
     <t xml:space="preserve">1015301</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 1 (front): unique P/N, matches the seat-frame assembly drawing and TU-530 Rev A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One P/N covers both front corners</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pre-fitted screw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ships installed by the supplier, correct screw and orientation</t>
+    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 1 (front) = bare connector 1012553 + screw 1012919, assembled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One assembly P/N covers both front corners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Component: bare connector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unchanged shared component inside the assembly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same piece as today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Component: screw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-fitted by the supplier per the assembly drawing</t>
   </si>
   <si>
     <t xml:space="preserve">Spec to be validated by Engineering before release</t>
@@ -142,16 +163,16 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
-    <t xml:space="preserve">[Drawing]  Corrected connector drawing: P/N 1015301 with fitted-screw callout (supersedes 1012553)</t>
+    <t xml:space="preserve">[Drawing]  Assembly drawing for 1015301 (front config): BOMs 1012553 + screw 1012919, with the fitted-screw callout</t>
   </si>
   <si>
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">[BOM]  Meritage BOM update: front connector line becomes 1015301, qty 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction (Vietnam): order by config P/N, pre-fit screw 1012919</t>
+    <t xml:space="preserve">[BOM]  Meritage product BOM update: front connector line reads assembly 1015301, qty 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction (Vietnam): order by ASSEMBLY P/N 1015301, pre-fit screw 1012919</t>
   </si>
   <si>
     <t xml:space="preserve">[Engineering]  Engineering validation of screw 1012919 as the released spec</t>
@@ -160,19 +181,22 @@
     <t xml:space="preserve">BRANCH 2 · BACK LEFT CONNECTOR   ·   Config 2 (back left, orientation-specific)</t>
   </si>
   <si>
-    <t xml:space="preserve">(shared P/N)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Back-left and back-right SHARE one part number today; drawings show wrong P/N 1012553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The two back configurations are physically different but undistinguished</t>
+    <t xml:space="preserve">Same shared connector piece; correct and unchanged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK as-is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Back-left and back-right arrive as ONE undistinguished assembly with screw 1012934, orientation random</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No left-specific assembly P/N exists to order</t>
   </si>
   <si>
     <t xml:space="preserve">1012934</t>
   </si>
   <si>
-    <t xml:space="preserve">Arrives installed; wrong, operator swaps it</t>
+    <t xml:space="preserve">Installed by the supplier; wrong, operator swaps it</t>
   </si>
   <si>
     <t xml:space="preserve">Part of the 11:40/unit rework</t>
@@ -193,7 +217,7 @@
     <t xml:space="preserve">n/a</t>
   </si>
   <si>
-    <t xml:space="preserve">About half the back connectors arrive with the screw-entry side wrong and are flipped by hand</t>
+    <t xml:space="preserve">About half arrive with the screw-entry side wrong and are flipped by hand</t>
   </si>
   <si>
     <t xml:space="preserve">-</t>
@@ -205,25 +229,25 @@
     <t xml:space="preserve">1015302</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 2 (back LEFT): unique P/N with the left orientation explicitly defined</t>
+    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 2 (back LEFT) = bare connector 1012553 + screw 40204, LEFT orientation</t>
   </si>
   <si>
     <t xml:space="preserve">Qty 1 per unit</t>
   </si>
   <si>
-    <t xml:space="preserve">Ships installed, correct left orientation</t>
+    <t xml:space="preserve">Pre-fitted in the LEFT orientation per the assembly drawing</t>
   </si>
   <si>
     <t xml:space="preserve">Spec to be validated by Engineering</t>
   </si>
   <si>
-    <t xml:space="preserve">[Drawing]  New connector drawing for 1015302 with LEFT orientation defined and screw callout (supersedes 1012553)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[BOM]  Meritage BOM update: back-left line becomes 1015302, qty 1 (split from the shared back P/N)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: pre-fit screw 40204 in left orientation</t>
+    <t xml:space="preserve">[Drawing]  Assembly drawing for 1015302 (back left): BOMs 1012553 + screw 40204 with the LEFT orientation defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[BOM]  Meritage product BOM update: back-left line reads assembly 1015302, qty 1 (split from the shared back line)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: order by ASSEMBLY P/N 1015302, pre-fit 40204 in left orientation</t>
   </si>
   <si>
     <t xml:space="preserve">[Engineering]  Engineering validation of screw 40204 as the released spec</t>
@@ -232,13 +256,10 @@
     <t xml:space="preserve">BRANCH 3 · BACK RIGHT CONNECTOR   ·   Config 3 (back right, orientation-specific)</t>
   </si>
   <si>
-    <t xml:space="preserve">Shares a part number with back-left today; drawings show wrong P/N 1012553</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Undistinguished from back-left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">About half arrive with the screw-entry side wrong and are flipped by hand</t>
+    <t xml:space="preserve">Arrives undistinguished from back-left, screw 1012934, orientation random</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No right-specific assembly P/N exists to order</t>
   </si>
   <si>
     <t xml:space="preserve">Pure rework</t>
@@ -247,22 +268,22 @@
     <t xml:space="preserve">1016592</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 3 (back RIGHT): unique P/N with the right orientation explicitly defined</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ships installed, correct right orientation</t>
+    <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 3 (back RIGHT) = bare connector 1012553 + screw 40204, RIGHT orientation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-fitted in the RIGHT orientation per the assembly drawing</t>
   </si>
   <si>
     <t xml:space="preserve">Same validation as back-left</t>
   </si>
   <si>
-    <t xml:space="preserve">[Drawing]  New connector drawing for 1016592 with RIGHT orientation defined and screw callout (supersedes 1012553)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[BOM]  Meritage BOM update: back-right line becomes 1016592, qty 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: pre-fit screw 40204 in right orientation</t>
+    <t xml:space="preserve">[Drawing]  Assembly drawing for 1016592 (back right): BOMs 1012553 + screw 40204 with the RIGHT orientation defined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[BOM]  Meritage product BOM update: back-right line reads assembly 1016592, qty 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: order by ASSEMBLY P/N 1016592, pre-fit 40204 in right orientation</t>
   </si>
   <si>
     <t xml:space="preserve">[Engineering]  Engineering validation of screw 40204 (shared with back-left, one validation covers both)</t>
@@ -875,7 +896,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1041,247 +1062,247 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="C16" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B18" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C18" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D18" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E18" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="13" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>2</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25" t="s">
-        <v>41</v>
+      <c r="B23" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C24" s="24"/>
       <c r="D24" s="24"/>
       <c r="E24" s="25"/>
       <c r="F24" s="25" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C25" s="24"/>
       <c r="D25" s="24"/>
       <c r="E25" s="25"/>
       <c r="F25" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="B27" s="26"/>
-      <c r="C27" s="26"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B31" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="C31" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="D31" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E31" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="F31" s="13" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E31" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="16" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>53</v>
@@ -1295,446 +1316,566 @@
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="15" t="s">
+      <c r="B35" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="22"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="25"/>
+      <c r="F44" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="C45" s="24"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C46" s="24"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="B49" s="27"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="27"/>
+      <c r="E49" s="27"/>
+      <c r="F49" s="27"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D52" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C53" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E53" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="16" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C54" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="D54" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="E54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17" t="s">
+    <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
+      <c r="C55" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D55" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E55" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C56" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="F56" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B58" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C58" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D58" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E58" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B36" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="20" t="s">
+      <c r="F58" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="D59" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C60" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E60" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B61" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C61" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="D36" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="E36" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="n">
+      <c r="D61" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="E61" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="21" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B62" s="22"/>
+      <c r="C62" s="22"/>
+      <c r="D62" s="22"/>
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F63" s="13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B64" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C64" s="24"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B37" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D37" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="E37" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="21" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B38" s="22"/>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="22"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B40" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C41" s="24"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="23" t="n">
+      <c r="B65" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C65" s="24"/>
+      <c r="D65" s="24"/>
+      <c r="E65" s="25"/>
+      <c r="F65" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B42" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="24"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="23" t="n">
+      <c r="B66" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="C66" s="24"/>
+      <c r="D66" s="24"/>
+      <c r="E66" s="25"/>
+      <c r="F66" s="25" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B43" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="C43" s="24"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="27" t="s">
-        <v>69</v>
-      </c>
-      <c r="B45" s="27"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="27"/>
-      <c r="E45" s="27"/>
-      <c r="F45" s="27"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B46" s="11"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B47" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B48" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C48" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D48" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="E48" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C49" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D49" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E49" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="16" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B50" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C50" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="D50" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="E50" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B51" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="C51" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D51" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="F51" s="16" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B53" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" s="13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B54" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="C54" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="E54" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="21" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B55" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C55" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D55" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="E55" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B56" s="22"/>
-      <c r="C56" s="22"/>
-      <c r="D56" s="22"/>
-      <c r="E56" s="22"/>
-      <c r="F56" s="22"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B57" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F57" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B58" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="C58" s="24"/>
-      <c r="D58" s="24"/>
-      <c r="E58" s="25"/>
-      <c r="F58" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B59" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="C59" s="24"/>
-      <c r="D59" s="24"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B60" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="C60" s="24"/>
-      <c r="D60" s="24"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="B61" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="C61" s="24"/>
-      <c r="D61" s="24"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25" t="s">
-        <v>41</v>
+      <c r="B67" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C67" s="24"/>
+      <c r="D67" s="24"/>
+      <c r="E67" s="25"/>
+      <c r="F67" s="25" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1744,31 +1885,31 @@
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="B43:D43"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B67:D67"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Connector workbook: CSI current state (1015301 x2 correct; split 1015302 x2 into 1015302 + new 1016592)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019MdxDfxB8wg2Ht2aZSuwqK
</commit_message>
<xml_diff>
--- a/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
+++ b/standard-work/docs/Meritage_Connector_BOM_Rework.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="95">
   <si>
     <t xml:space="preserve">MERITAGE FLAT CONNECTOR SYSTEM · BOM REWORK BY BRANCH</t>
   </si>
   <si>
-    <t xml:space="preserve">How to read this: 1012553 is the BARE connector piece (shared component, used in every position, unchanged). The differentiation happens one level up, at the ASSEMBLY: bare connector + the right screw + the right orientation = three distinct assemblies (1015301 front, 1015302 back-left, 1016592 back-right). Today the supplier effectively ships ONE generic assembly, so the line swaps screws and flips orientation by hand. Scope: define and order the three assemblies, 07/2026.</t>
+    <t xml:space="preserve">How to read this: 1012553 is the BARE connector piece (shared component in every position, unchanged). Differentiation happens at the ASSEMBLY level: bare connector + the right screw + the right orientation. CSI TODAY: 1015301 qty 2 (front) and 1015302 qty 2 (BOTH backs). The front line is already correct. The defect is the back line: two different connectors (left / right) share 1015302. Fix: split it (1015302 back-left qty 1, ADD 1016592 back-right qty 1) and define all three assemblies with their pre-fitted screws so Vietnam ships them ready, 07/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Labor recovered per unit (min)</t>
@@ -79,16 +79,28 @@
     <t xml:space="preserve">OK as-is: the shared base component</t>
   </si>
   <si>
+    <t xml:space="preserve">CSI BOM line (today)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1015301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSI already shows 1015301 qty 2 for the fronts: the P/N structure here is CORRECT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No BOM change needed on the front line</t>
+  </si>
+  <si>
     <t xml:space="preserve">Assembly, as shipped</t>
   </si>
   <si>
     <t xml:space="preserve">(generic)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supplier assembles the bare connector with screw 40200; no front-specific assembly P/N is ordered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The generic assembly is what forces the rework</t>
+    <t xml:space="preserve">What actually arrives is assembled with screw 40200; the 1015301 assembly content is not defined/enforced at the supplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The undefined assembly content is what forces the rework</t>
   </si>
   <si>
     <t xml:space="preserve">Screw, as shipped</t>
@@ -124,9 +136,6 @@
     <t xml:space="preserve">Connector ASSEMBLY</t>
   </si>
   <si>
-    <t xml:space="preserve">1015301</t>
-  </si>
-  <si>
     <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 1 (front) = bare connector 1012553 + screw 1012919, assembled</t>
   </si>
   <si>
@@ -169,7 +178,7 @@
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">[BOM]  Meritage product BOM update: front connector line reads assembly 1015301, qty 2</t>
+    <t xml:space="preserve">[BOM]  CSI: no structural change on the front line (already 1015301 qty 2); confirm it points at the new assembly definition</t>
   </si>
   <si>
     <t xml:space="preserve">[Procurement]  Supplier PO + work instruction (Vietnam): order by ASSEMBLY P/N 1015301, pre-fit screw 1012919</t>
@@ -187,10 +196,19 @@
     <t xml:space="preserve">OK as-is</t>
   </si>
   <si>
-    <t xml:space="preserve">Back-left and back-right arrive as ONE undistinguished assembly with screw 1012934, orientation random</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No left-specific assembly P/N exists to order</t>
+    <t xml:space="preserve">1015302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSI shows 1015302 qty 2 covering BOTH backs, even though back-left and back-right are different parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is the line that must be split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrives assembled with screw 1012934, orientation random between left and right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Undistinguished assembly content</t>
   </si>
   <si>
     <t xml:space="preserve">1012934</t>
@@ -226,9 +244,6 @@
     <t xml:space="preserve">Pure rework, zero value added</t>
   </si>
   <si>
-    <t xml:space="preserve">1015302</t>
-  </si>
-  <si>
     <t xml:space="preserve">ASSY MER HORZ CONNECTOR Config 2 (back LEFT) = bare connector 1012553 + screw 40204, LEFT orientation</t>
   </si>
   <si>
@@ -244,7 +259,7 @@
     <t xml:space="preserve">[Drawing]  Assembly drawing for 1015302 (back left): BOMs 1012553 + screw 40204 with the LEFT orientation defined</t>
   </si>
   <si>
-    <t xml:space="preserve">[BOM]  Meritage product BOM update: back-left line reads assembly 1015302, qty 1 (split from the shared back line)</t>
+    <t xml:space="preserve">[BOM]  CSI: change 1015302 from qty 2 to qty 1 (back-LEFT only)</t>
   </si>
   <si>
     <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: order by ASSEMBLY P/N 1015302, pre-fit 40204 in left orientation</t>
@@ -256,12 +271,15 @@
     <t xml:space="preserve">BRANCH 3 · BACK RIGHT CONNECTOR   ·   Config 3 (back right, orientation-specific)</t>
   </si>
   <si>
+    <t xml:space="preserve">Back-right is currently buried inside the shared 1015302 qty-2 line; 1016592 is NOT in the CSI BOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The missing P/N: this is the core CSI defect</t>
+  </si>
+  <si>
     <t xml:space="preserve">Arrives undistinguished from back-left, screw 1012934, orientation random</t>
   </si>
   <si>
-    <t xml:space="preserve">No right-specific assembly P/N exists to order</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pure rework</t>
   </si>
   <si>
@@ -280,7 +298,7 @@
     <t xml:space="preserve">[Drawing]  Assembly drawing for 1016592 (back right): BOMs 1012553 + screw 40204 with the RIGHT orientation defined</t>
   </si>
   <si>
-    <t xml:space="preserve">[BOM]  Meritage product BOM update: back-right line reads assembly 1016592, qty 1</t>
+    <t xml:space="preserve">[BOM]  CSI: ADD line 1016592 qty 1 (back-RIGHT); create the P/N in CSI if it does not exist yet</t>
   </si>
   <si>
     <t xml:space="preserve">[Procurement]  Supplier PO + work instruction: order by ASSEMBLY P/N 1016592, pre-fit 40204 in right orientation</t>
@@ -896,7 +914,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1082,65 +1100,65 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
+      <c r="C17" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B19" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C19" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D19" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="21" t="s">
+      <c r="F19" s="13" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>37</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D20" s="19" t="s">
         <v>38</v>
@@ -1154,13 +1172,13 @@
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>40</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D21" s="19" t="s">
         <v>41</v>
@@ -1172,197 +1190,197 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
+    <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="C22" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="21" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25" t="s">
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13" t="s">
         <v>48</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C25" s="24"/>
       <c r="D25" s="24"/>
       <c r="E25" s="25"/>
       <c r="F25" s="25" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C26" s="24"/>
       <c r="D26" s="24"/>
       <c r="E26" s="25"/>
       <c r="F26" s="25" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C27" s="24"/>
       <c r="D27" s="24"/>
       <c r="E27" s="25"/>
       <c r="F27" s="25" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B32" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C32" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D32" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E32" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F32" s="13" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="E32" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E33" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E34" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>61</v>
@@ -1376,506 +1394,566 @@
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B36" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="E36" s="14" t="s">
+      <c r="B37" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="F36" s="16" t="s">
+      <c r="D37" s="15" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
+      <c r="E37" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F38" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B40" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C40" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D40" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="12" t="s">
+      <c r="E40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F38" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" s="20" t="s">
-        <v>68</v>
-      </c>
-      <c r="D39" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E39" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="B40" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="E40" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="21" t="s">
-        <v>39</v>
+      <c r="F40" s="13" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="E41" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="21" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E42" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C41" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D41" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="E41" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="22" t="s">
+      <c r="B43" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12" t="s">
+      <c r="C43" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="D43" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E43" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B43" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="C44" s="24"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25" t="s">
+      <c r="B45" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C45" s="24"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="25"/>
-      <c r="F45" s="25" t="s">
-        <v>48</v>
+      <c r="F45" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C46" s="24"/>
       <c r="D46" s="24"/>
       <c r="E46" s="25"/>
       <c r="F46" s="25" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B47" s="24" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C47" s="24"/>
       <c r="D47" s="24"/>
       <c r="E47" s="25"/>
       <c r="F47" s="25" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="27" t="s">
-        <v>77</v>
-      </c>
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-      <c r="E49" s="27"/>
-      <c r="F49" s="27"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" s="24"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="25"/>
+      <c r="F48" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" s="24"/>
+      <c r="D49" s="24"/>
+      <c r="E49" s="25"/>
+      <c r="F49" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12" t="s">
+      <c r="B52" s="11"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B51" s="13" t="s">
+      <c r="B53" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C51" s="13" t="s">
+      <c r="C53" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="D53" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E51" s="12" t="s">
+      <c r="E53" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F51" s="13" t="s">
+      <c r="F53" s="13" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B52" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C52" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D52" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="E52" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="16" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D53" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E53" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="16" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C54" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D54" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="16" t="s">
         <v>57</v>
-      </c>
-      <c r="D54" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E54" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="16" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
       <c r="E55" s="14" t="n">
         <v>1</v>
       </c>
       <c r="F55" s="16" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C56" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E56" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E57" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B56" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C56" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D56" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="E56" s="14" t="s">
+      <c r="B58" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C58" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="F56" s="16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B57" s="17"/>
-      <c r="C57" s="17"/>
-      <c r="D57" s="17"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="s">
+      <c r="D58" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E58" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B59" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E59" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F59" s="16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B60" s="17"/>
+      <c r="C60" s="17"/>
+      <c r="D60" s="17"/>
+      <c r="E60" s="17"/>
+      <c r="F60" s="17"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B58" s="13" t="s">
+      <c r="B61" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C58" s="13" t="s">
+      <c r="C61" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D58" s="13" t="s">
+      <c r="D61" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="E58" s="12" t="s">
+      <c r="E61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F58" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B59" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D59" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="E59" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="18" t="n">
+      <c r="F61" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B62" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C62" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="D62" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E62" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="21" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B60" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C60" s="20" t="s">
+      <c r="B63" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C63" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D60" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="E60" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" s="21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="18" t="n">
+      <c r="D63" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B61" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C61" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D61" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="E61" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="21" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="22" t="s">
+      <c r="B64" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B62" s="22"/>
-      <c r="C62" s="22"/>
-      <c r="D62" s="22"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="12" t="s">
+      <c r="C64" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="D64" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="E64" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B65" s="22"/>
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="22"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B63" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C63" s="13"/>
-      <c r="D63" s="13"/>
-      <c r="E63" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F63" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B64" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="25" t="s">
+      <c r="B66" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="65" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B65" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="C65" s="24"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="25"/>
-      <c r="F65" s="25" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B66" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="25"/>
-      <c r="F66" s="25" t="s">
-        <v>48</v>
+      <c r="F66" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B67" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C67" s="24"/>
       <c r="D67" s="24"/>
       <c r="E67" s="25"/>
       <c r="F67" s="25" t="s">
-        <v>48</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B68" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="C68" s="24"/>
+      <c r="D68" s="24"/>
+      <c r="E68" s="25"/>
+      <c r="F68" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B69" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C69" s="24"/>
+      <c r="D69" s="24"/>
+      <c r="E69" s="25"/>
+      <c r="F69" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B70" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="C70" s="24"/>
+      <c r="D70" s="24"/>
+      <c r="E70" s="25"/>
+      <c r="F70" s="25" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1885,31 +1963,31 @@
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B46:D46"/>
     <mergeCell ref="B47:D47"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A65:F65"/>
     <mergeCell ref="B66:D66"/>
     <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="B70:D70"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>